<commit_message>
Updated the End to End test cases
</commit_message>
<xml_diff>
--- a/test-cases/test-cases.xlsx
+++ b/test-cases/test-cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1098" uniqueCount="631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1109" uniqueCount="640">
   <si>
     <t>TC ID</t>
   </si>
@@ -1310,6 +1310,33 @@
   </si>
   <si>
     <t>A surcharge gives a higher premium than no modifier, and a discount gives a lower one. The exact adjustment is: Configured rule / requirement to confirm.</t>
+  </si>
+  <si>
+    <t>TC-073</t>
+  </si>
+  <si>
+    <t>Login, Bond Creation, Logout</t>
+  </si>
+  <si>
+    <t>End-to-end: login, change language, drag and drop an attachment, logout, and see the Tinubu logo</t>
+  </si>
+  <si>
+    <t>E2E</t>
+  </si>
+  <si>
+    <t>User is on the Login page; QA bond 09182606481644270732 exists; valid QA credentials in environment variables</t>
+  </si>
+  <si>
+    <t>Valid username + valid password; language Italiano, then English (US); a generated text file qa-e2e-&lt;timestamp&gt;.txt; attachment category Misc</t>
+  </si>
+  <si>
+    <t>1. Sign in with the QA account. 2. In the navbar, change Language to Italiano. 3. Change Language back to English (US). 4. Search for bond 09182606481644270732 and open it. 5. Click Add under attachments. 6. Drag the file onto the dropzone. 7. Choose category Misc and click Save. 8. Reload the bond page. 9. Log out from the profile menu. 10. Check the Sign In page.</t>
+  </si>
+  <si>
+    <t>The dashboard loads after sign-in. The page language changes to it-IT and back to en-US. The dropped file is listed in the dialog, Save returns 201, and the file is listed on the bond after reload. After logout the Sign In page is shown, its title contains Sign In, and the Tinubu logo image is loaded.</t>
+  </si>
+  <si>
+    <t>2026-09-29 automated run: every step passed; the language returned to English (US) and the attachment was listed on bond 1008565 after reload.</t>
   </si>
   <si>
     <t>S-01</t>
@@ -2315,7 +2342,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -4831,31 +4858,31 @@
         <v>433</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>124</v>
+        <v>434</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="I73" s="2" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="J73" s="2" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K73" s="2" t="s">
         <v>21</v>
@@ -4863,34 +4890,34 @@
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>12</v>
+        <v>124</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>289</v>
+        <v>444</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>17</v>
+        <v>446</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="I74" s="2" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="J74" s="2" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="K74" s="2" t="s">
         <v>21</v>
@@ -4898,13 +4925,13 @@
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>124</v>
+        <v>12</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>289</v>
@@ -4913,19 +4940,19 @@
         <v>15</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>450</v>
+        <v>17</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="I75" s="2" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="J75" s="2" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="K75" s="2" t="s">
         <v>21</v>
@@ -4933,16 +4960,16 @@
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>455</v>
+        <v>124</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>457</v>
+        <v>289</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>15</v>
@@ -4971,31 +4998,31 @@
         <v>463</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="I77" s="2" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="J77" s="2" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="K77" s="2" t="s">
         <v>21</v>
@@ -5003,314 +5030,314 @@
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>124</v>
+        <v>464</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="I78" s="2" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="J78" s="2" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="K78" s="2" t="s">
-        <v>81</v>
+        <v>21</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>124</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="H79" s="2" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="I79" s="2" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="J79" s="2" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="K79" s="2" t="s">
-        <v>21</v>
+        <v>81</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>12</v>
+        <v>124</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="I80" s="2" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="J80" s="2" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="K80" s="2" t="s">
-        <v>81</v>
+        <v>21</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>436</v>
+        <v>494</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="I81" s="2" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="J81" s="2" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="K81" s="2" t="s">
-        <v>496</v>
+        <v>81</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>458</v>
+        <v>445</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="I82" s="2" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="J82" s="2" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="K82" s="2" t="s">
-        <v>496</v>
+        <v>505</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
       <c r="G83" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="H83" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="I83" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="J83" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="K83" s="2" t="s">
         <v>505</v>
-      </c>
-      <c r="H83" s="2" t="s">
-        <v>506</v>
-      </c>
-      <c r="I83" s="2" t="s">
-        <v>507</v>
-      </c>
-      <c r="J83" s="2" t="s">
-        <v>508</v>
-      </c>
-      <c r="K83" s="2" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="H84" s="2" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="I84" s="2" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="J84" s="2" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="K84" s="2" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>517</v>
+        <v>466</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>518</v>
+        <v>467</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="H85" s="2" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="I85" s="2" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="J85" s="2" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="K85" s="2" t="s">
-        <v>81</v>
+        <v>21</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>124</v>
+        <v>12</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>517</v>
+        <v>526</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="I86" s="2" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="J86" s="2" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="K86" s="2" t="s">
         <v>81</v>
@@ -5318,69 +5345,69 @@
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>12</v>
+        <v>124</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>532</v>
+        <v>526</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="H87" s="2" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="I87" s="2" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="J87" s="2" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="K87" s="2" t="s">
-        <v>21</v>
+        <v>81</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>124</v>
+        <v>12</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>532</v>
+        <v>541</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>436</v>
+        <v>542</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="H88" s="2" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="I88" s="2" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J88" s="2" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K88" s="2" t="s">
         <v>21</v>
@@ -5388,34 +5415,34 @@
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>12</v>
+        <v>124</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>532</v>
+        <v>541</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>546</v>
+        <v>445</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="H89" s="2" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="I89" s="2" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="J89" s="2" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="K89" s="2" t="s">
         <v>21</v>
@@ -5423,69 +5450,69 @@
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>532</v>
+        <v>541</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="I90" s="2" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="J90" s="2" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="K90" s="2" t="s">
-        <v>67</v>
+        <v>21</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>124</v>
+        <v>12</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>560</v>
+        <v>541</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>436</v>
+        <v>562</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="I91" s="2" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="J91" s="2" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="K91" s="2" t="s">
         <v>67</v>
@@ -5493,34 +5520,34 @@
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>124</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>560</v>
+        <v>569</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>478</v>
+        <v>445</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="H92" s="2" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="I92" s="2" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="J92" s="2" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="K92" s="2" t="s">
         <v>67</v>
@@ -5528,34 +5555,34 @@
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>124</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>560</v>
+        <v>569</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>573</v>
+        <v>55</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>478</v>
+        <v>487</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="I93" s="2" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="J93" s="2" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="K93" s="2" t="s">
         <v>67</v>
@@ -5563,34 +5590,34 @@
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>124</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>560</v>
+        <v>569</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>478</v>
+        <v>487</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>421</v>
+        <v>584</v>
       </c>
       <c r="I94" s="2" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="J94" s="2" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="K94" s="2" t="s">
         <v>67</v>
@@ -5598,34 +5625,34 @@
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>124</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>560</v>
+        <v>569</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>478</v>
+        <v>487</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>586</v>
+        <v>421</v>
       </c>
       <c r="I95" s="2" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="J95" s="2" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="K95" s="2" t="s">
         <v>67</v>
@@ -5633,22 +5660,22 @@
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>590</v>
+        <v>124</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>592</v>
+        <v>569</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>15</v>
+        <v>582</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>593</v>
+        <v>487</v>
       </c>
       <c r="G96" s="2" t="s">
         <v>594</v>
@@ -5671,136 +5698,136 @@
         <v>598</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>12</v>
+        <v>599</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>458</v>
+        <v>602</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="H97" s="2" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="I97" s="2" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="J97" s="2" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="K97" s="2" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>124</v>
+        <v>12</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>600</v>
+        <v>609</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>436</v>
+        <v>467</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="H98" s="2" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="I98" s="2" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="J98" s="2" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="K98" s="2" t="s">
-        <v>496</v>
+        <v>21</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>590</v>
+        <v>124</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>600</v>
+        <v>609</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>613</v>
+        <v>445</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="H99" s="2" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="I99" s="2" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="J99" s="2" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="K99" s="2" t="s">
-        <v>67</v>
+        <v>505</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>590</v>
+        <v>599</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>620</v>
+        <v>609</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>614</v>
+        <v>623</v>
       </c>
       <c r="H100" s="2" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="I100" s="2" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="J100" s="2" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="K100" s="2" t="s">
         <v>67</v>
@@ -5808,36 +5835,71 @@
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>590</v>
+        <v>599</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>592</v>
+        <v>629</v>
       </c>
       <c r="E101" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="G101" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="H101" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="I101" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="J101" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="K101" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A102" s="2" t="s">
+        <v>634</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="E102" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="F101" s="2" t="s">
-        <v>613</v>
-      </c>
-      <c r="G101" s="2" t="s">
-        <v>627</v>
-      </c>
-      <c r="H101" s="2" t="s">
-        <v>628</v>
-      </c>
-      <c r="I101" s="2" t="s">
-        <v>629</v>
-      </c>
-      <c r="J101" s="2" t="s">
-        <v>630</v>
-      </c>
-      <c r="K101" s="2" t="s">
+      <c r="F102" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="G102" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="H102" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="I102" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="J102" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="K102" s="2" t="s">
         <v>67</v>
       </c>
     </row>
@@ -5852,6 +5914,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>